<commit_message>
Began analysis of bird survey data. Mostly spent time generating presence absence summaries and visualising trends between sites, habitats and survey methods.
</commit_message>
<xml_diff>
--- a/birdsurvey_data/phase2_BirdSurveys.xlsx
+++ b/birdsurvey_data/phase2_BirdSurveys.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charl\Documents\University\Year 5 Masters\Research Project\2. Analysis\final_research_project\birdsurvey_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E885BACE-B40F-4839-812E-01539A5103FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7FE38D-BF1C-4856-B419-0466786526F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BD219C88-E6CD-40D9-A547-1ACB8E76B1AE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="46">
   <si>
     <t>site</t>
   </si>
@@ -81,9 +81,6 @@
   </si>
   <si>
     <t>seen</t>
-  </si>
-  <si>
-    <t>grassland</t>
   </si>
   <si>
     <t>moorland</t>
@@ -594,7 +591,7 @@
         <v>12</v>
       </c>
       <c r="I1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -617,7 +614,7 @@
         <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H2" t="s">
         <v>13</v>
@@ -646,7 +643,7 @@
         <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H3" t="s">
         <v>13</v>
@@ -675,7 +672,7 @@
         <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H4" t="s">
         <v>13</v>
@@ -704,7 +701,7 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H5" t="s">
         <v>13</v>
@@ -733,7 +730,7 @@
         <v>11</v>
       </c>
       <c r="G6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H6" t="s">
         <v>13</v>
@@ -762,7 +759,7 @@
         <v>11</v>
       </c>
       <c r="G7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H7" t="s">
         <v>13</v>
@@ -791,10 +788,10 @@
         <v>11</v>
       </c>
       <c r="G8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I8" t="b">
         <v>0</v>
@@ -820,7 +817,7 @@
         <v>11</v>
       </c>
       <c r="G9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H9" t="s">
         <v>13</v>
@@ -849,10 +846,10 @@
         <v>11</v>
       </c>
       <c r="G10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I10" t="b">
         <v>0</v>
@@ -878,7 +875,7 @@
         <v>11</v>
       </c>
       <c r="G11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H11" t="s">
         <v>13</v>
@@ -907,7 +904,7 @@
         <v>9</v>
       </c>
       <c r="G12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H12" t="s">
         <v>13</v>
@@ -936,7 +933,7 @@
         <v>9</v>
       </c>
       <c r="G13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H13" t="s">
         <v>13</v>
@@ -965,7 +962,7 @@
         <v>9</v>
       </c>
       <c r="G14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H14" t="s">
         <v>14</v>
@@ -994,7 +991,7 @@
         <v>9</v>
       </c>
       <c r="G15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H15" t="s">
         <v>14</v>
@@ -1023,7 +1020,7 @@
         <v>9</v>
       </c>
       <c r="G16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H16" t="s">
         <v>13</v>
@@ -1049,10 +1046,10 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H17" t="s">
         <v>13</v>
@@ -1078,10 +1075,10 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H18" t="s">
         <v>14</v>
@@ -1107,10 +1104,10 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H19" t="s">
         <v>13</v>
@@ -1136,10 +1133,10 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H20" t="s">
         <v>13</v>
@@ -1165,10 +1162,10 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H21" t="s">
         <v>13</v>
@@ -1194,10 +1191,10 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H22" t="s">
         <v>13</v>
@@ -1223,10 +1220,10 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H23" t="s">
         <v>13</v>
@@ -1252,10 +1249,10 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H24" t="s">
         <v>13</v>
@@ -1281,10 +1278,10 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F25" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H25" t="s">
         <v>13</v>
@@ -1310,10 +1307,10 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G26" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H26" t="s">
         <v>13</v>
@@ -1339,10 +1336,10 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F27" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G27" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H27" t="s">
         <v>13</v>
@@ -1368,10 +1365,10 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F28" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H28" t="s">
         <v>14</v>
@@ -1397,13 +1394,13 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F29" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G29" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H29" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I29" t="b">
         <v>0</v>
@@ -1426,10 +1423,10 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F30" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G30" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H30" t="s">
         <v>14</v>
@@ -1455,13 +1452,13 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F31" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G31" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H31" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I31" t="b">
         <v>0</v>
@@ -1484,7 +1481,7 @@
         <v>0.40972222222222221</v>
       </c>
       <c r="F32" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
@@ -1507,10 +1504,10 @@
         <v>10</v>
       </c>
       <c r="G33" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H33" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I33" t="b">
         <v>0</v>
@@ -1536,7 +1533,7 @@
         <v>10</v>
       </c>
       <c r="G34" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H34" t="s">
         <v>14</v>
@@ -1565,7 +1562,7 @@
         <v>10</v>
       </c>
       <c r="G35" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H35" t="s">
         <v>14</v>
@@ -1594,7 +1591,7 @@
         <v>10</v>
       </c>
       <c r="G36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H36" t="s">
         <v>14</v>
@@ -1623,7 +1620,7 @@
         <v>10</v>
       </c>
       <c r="G37" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H37" t="s">
         <v>14</v>
@@ -1652,7 +1649,7 @@
         <v>10</v>
       </c>
       <c r="G38" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H38" t="s">
         <v>14</v>
@@ -1681,7 +1678,7 @@
         <v>10</v>
       </c>
       <c r="G39" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H39" t="s">
         <v>14</v>
@@ -1710,7 +1707,7 @@
         <v>10</v>
       </c>
       <c r="G40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H40" t="s">
         <v>14</v>
@@ -1739,7 +1736,7 @@
         <v>10</v>
       </c>
       <c r="G41" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H41" t="s">
         <v>14</v>
@@ -1768,7 +1765,7 @@
         <v>10</v>
       </c>
       <c r="G42" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H42" t="s">
         <v>14</v>
@@ -1797,7 +1794,7 @@
         <v>11</v>
       </c>
       <c r="G43" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H43" t="s">
         <v>14</v>
@@ -1826,10 +1823,10 @@
         <v>9</v>
       </c>
       <c r="G44" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H44" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I44" t="b">
         <v>0</v>
@@ -1855,10 +1852,10 @@
         <v>9</v>
       </c>
       <c r="G45" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H45" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I45" t="b">
         <v>0</v>
@@ -1881,7 +1878,7 @@
         <v>0.44444444444444398</v>
       </c>
       <c r="F46" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
@@ -1901,10 +1898,10 @@
         <v>0.44444444444444398</v>
       </c>
       <c r="F47" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G47" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H47" t="s">
         <v>14</v>
@@ -1930,10 +1927,10 @@
         <v>0.44444444444444398</v>
       </c>
       <c r="F48" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G48" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H48" t="s">
         <v>14</v>
@@ -1944,10 +1941,10 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B49" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C49" s="1">
         <v>45841</v>
@@ -1962,7 +1959,7 @@
         <v>10</v>
       </c>
       <c r="G49" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H49" t="s">
         <v>13</v>
@@ -1973,10 +1970,10 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B50" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C50" s="1">
         <v>45841</v>
@@ -1991,7 +1988,7 @@
         <v>10</v>
       </c>
       <c r="G50" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H50" t="s">
         <v>13</v>
@@ -2002,10 +1999,10 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B51" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C51" s="1">
         <v>45841</v>
@@ -2020,7 +2017,7 @@
         <v>11</v>
       </c>
       <c r="G51" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H51" t="s">
         <v>13</v>
@@ -2031,10 +2028,10 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B52" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C52" s="1">
         <v>45841</v>
@@ -2049,7 +2046,7 @@
         <v>11</v>
       </c>
       <c r="G52" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H52" t="s">
         <v>13</v>
@@ -2060,10 +2057,10 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B53" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C53" s="1">
         <v>45841</v>
@@ -2078,7 +2075,7 @@
         <v>11</v>
       </c>
       <c r="G53" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H53" t="s">
         <v>13</v>
@@ -2089,10 +2086,10 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B54" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C54" s="1">
         <v>45841</v>
@@ -2107,10 +2104,10 @@
         <v>9</v>
       </c>
       <c r="G54" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H54" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I54" t="b">
         <v>0</v>
@@ -2118,10 +2115,10 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B55" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C55" s="1">
         <v>45841</v>
@@ -2133,10 +2130,10 @@
         <v>0.5131944444444444</v>
       </c>
       <c r="F55" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G55" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H55" t="s">
         <v>14</v>
@@ -2147,10 +2144,10 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B56" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C56" s="1">
         <v>45841</v>
@@ -2162,13 +2159,13 @@
         <v>0.5131944444444444</v>
       </c>
       <c r="F56" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G56" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H56" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I56" t="b">
         <v>1</v>
@@ -2176,10 +2173,10 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B57" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C57" s="1">
         <v>45841</v>
@@ -2191,10 +2188,10 @@
         <v>0.5131944444444444</v>
       </c>
       <c r="F57" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G57" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H57" t="s">
         <v>14</v>
@@ -2205,10 +2202,10 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B58" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C58" s="1">
         <v>45841</v>
@@ -2220,13 +2217,13 @@
         <v>0.5131944444444444</v>
       </c>
       <c r="F58" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G58" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H58" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I58" t="b">
         <v>0</v>
@@ -2234,10 +2231,10 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B59" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C59" s="1">
         <v>45841</v>
@@ -2249,13 +2246,13 @@
         <v>0.5131944444444444</v>
       </c>
       <c r="F59" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G59" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H59" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I59" t="b">
         <v>0</v>
@@ -2263,10 +2260,10 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B60" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C60" s="1">
         <v>45841</v>
@@ -2278,10 +2275,10 @@
         <v>0.5131944444444444</v>
       </c>
       <c r="F60" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G60" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H60" t="s">
         <v>13</v>
@@ -2292,10 +2289,10 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B61" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C61" s="1">
         <v>45841</v>
@@ -2307,13 +2304,13 @@
         <v>0.5131944444444444</v>
       </c>
       <c r="F61" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G61" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H61" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I61" t="b">
         <v>0</v>
@@ -2321,10 +2318,10 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B62" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C62" s="1">
         <v>45841</v>
@@ -2336,13 +2333,13 @@
         <v>0.5131944444444444</v>
       </c>
       <c r="F62" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G62" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H62" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I62" t="b">
         <v>0</v>
@@ -2350,10 +2347,10 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B63" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C63" s="1">
         <v>45841</v>
@@ -2365,13 +2362,13 @@
         <v>0.5131944444444444</v>
       </c>
       <c r="F63" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G63" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H63" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I63" t="b">
         <v>0</v>
@@ -2379,10 +2376,10 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B64" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C64" s="1">
         <v>45841</v>
@@ -2394,10 +2391,10 @@
         <v>0.5131944444444444</v>
       </c>
       <c r="F64" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G64" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H64" t="s">
         <v>13</v>
@@ -2408,10 +2405,10 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B65" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C65" s="1">
         <v>45841</v>
@@ -2423,13 +2420,13 @@
         <v>0.5131944444444444</v>
       </c>
       <c r="F65" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G65" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H65" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I65" t="b">
         <v>0</v>
@@ -2437,10 +2434,10 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B66" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C66" s="1">
         <v>45841</v>
@@ -2452,10 +2449,10 @@
         <v>0.5131944444444444</v>
       </c>
       <c r="F66" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G66" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H66" t="s">
         <v>13</v>
@@ -2466,10 +2463,10 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B67" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C67" s="1">
         <v>45841</v>
@@ -2481,10 +2478,10 @@
         <v>0.5131944444444444</v>
       </c>
       <c r="F67" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G67" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H67" t="s">
         <v>13</v>
@@ -2495,10 +2492,10 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B68" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C68" s="1">
         <v>45841</v>
@@ -2510,12 +2507,12 @@
         <v>0.5131944444444444</v>
       </c>
       <c r="F68" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B69" t="s">
         <v>7</v>
@@ -2533,7 +2530,7 @@
         <v>10</v>
       </c>
       <c r="G69" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H69" t="s">
         <v>13</v>
@@ -2544,7 +2541,7 @@
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B70" t="s">
         <v>7</v>
@@ -2562,7 +2559,7 @@
         <v>10</v>
       </c>
       <c r="G70" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H70" t="s">
         <v>13</v>
@@ -2573,7 +2570,7 @@
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B71" t="s">
         <v>7</v>
@@ -2591,7 +2588,7 @@
         <v>10</v>
       </c>
       <c r="G71" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H71" t="s">
         <v>13</v>
@@ -2602,7 +2599,7 @@
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B72" t="s">
         <v>7</v>
@@ -2620,7 +2617,7 @@
         <v>10</v>
       </c>
       <c r="G72" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H72" t="s">
         <v>13</v>
@@ -2631,7 +2628,7 @@
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B73" t="s">
         <v>7</v>
@@ -2649,7 +2646,7 @@
         <v>11</v>
       </c>
       <c r="G73" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H73" t="s">
         <v>13</v>
@@ -2660,7 +2657,7 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B74" t="s">
         <v>7</v>
@@ -2678,7 +2675,7 @@
         <v>11</v>
       </c>
       <c r="G74" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H74" t="s">
         <v>13</v>
@@ -2689,7 +2686,7 @@
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B75" t="s">
         <v>7</v>
@@ -2707,7 +2704,7 @@
         <v>11</v>
       </c>
       <c r="G75" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H75" t="s">
         <v>13</v>
@@ -2718,7 +2715,7 @@
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B76" t="s">
         <v>7</v>
@@ -2736,7 +2733,7 @@
         <v>11</v>
       </c>
       <c r="G76" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H76" t="s">
         <v>13</v>
@@ -2747,7 +2744,7 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B77" t="s">
         <v>7</v>
@@ -2765,7 +2762,7 @@
         <v>9</v>
       </c>
       <c r="G77" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H77" t="s">
         <v>13</v>
@@ -2776,7 +2773,7 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B78" t="s">
         <v>7</v>
@@ -2791,10 +2788,10 @@
         <v>0.5625</v>
       </c>
       <c r="F78" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G78" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H78" t="s">
         <v>13</v>
@@ -2805,7 +2802,7 @@
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B79" t="s">
         <v>7</v>
@@ -2820,10 +2817,10 @@
         <v>0.5625</v>
       </c>
       <c r="F79" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G79" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H79" t="s">
         <v>13</v>
@@ -2834,7 +2831,7 @@
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B80" t="s">
         <v>7</v>
@@ -2849,13 +2846,13 @@
         <v>0.5625</v>
       </c>
       <c r="F80" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G80" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H80" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I80" t="b">
         <v>0</v>
@@ -2863,7 +2860,7 @@
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B81" t="s">
         <v>7</v>
@@ -2878,13 +2875,13 @@
         <v>0.5625</v>
       </c>
       <c r="F81" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G81" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H81" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I81" t="b">
         <v>0</v>
@@ -2892,7 +2889,7 @@
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B82" t="s">
         <v>7</v>
@@ -2907,13 +2904,13 @@
         <v>0.5625</v>
       </c>
       <c r="F82" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G82" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H82" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I82" t="b">
         <v>0</v>
@@ -2921,7 +2918,7 @@
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B83" t="s">
         <v>7</v>
@@ -2936,13 +2933,13 @@
         <v>0.5625</v>
       </c>
       <c r="F83" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G83" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H83" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I83" t="b">
         <v>0</v>
@@ -2950,7 +2947,7 @@
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B84" t="s">
         <v>7</v>
@@ -2965,13 +2962,13 @@
         <v>0.5625</v>
       </c>
       <c r="F84" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G84" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H84" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I84" t="b">
         <v>0</v>
@@ -2979,7 +2976,7 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B85" t="s">
         <v>7</v>
@@ -2994,10 +2991,10 @@
         <v>0.5625</v>
       </c>
       <c r="F85" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G85" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H85" t="s">
         <v>13</v>
@@ -3008,7 +3005,7 @@
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B86" t="s">
         <v>7</v>
@@ -3023,10 +3020,10 @@
         <v>0.5625</v>
       </c>
       <c r="F86" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G86" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H86" t="s">
         <v>13</v>
@@ -3037,7 +3034,7 @@
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B87" t="s">
         <v>7</v>
@@ -3052,10 +3049,10 @@
         <v>0.5625</v>
       </c>
       <c r="F87" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G87" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H87" t="s">
         <v>13</v>
@@ -3066,7 +3063,7 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B88" t="s">
         <v>7</v>
@@ -3081,10 +3078,10 @@
         <v>0.5625</v>
       </c>
       <c r="F88" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G88" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H88" t="s">
         <v>13</v>
@@ -3095,7 +3092,7 @@
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B89" t="s">
         <v>7</v>
@@ -3110,10 +3107,10 @@
         <v>0.5625</v>
       </c>
       <c r="F89" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G89" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H89" t="s">
         <v>13</v>
@@ -3124,7 +3121,7 @@
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B90" t="s">
         <v>7</v>
@@ -3139,10 +3136,10 @@
         <v>0.5625</v>
       </c>
       <c r="F90" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G90" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H90" t="s">
         <v>13</v>
@@ -3153,7 +3150,7 @@
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B91" t="s">
         <v>7</v>
@@ -3168,10 +3165,10 @@
         <v>0.5625</v>
       </c>
       <c r="F91" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G91" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H91" t="s">
         <v>13</v>
@@ -3182,7 +3179,7 @@
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B92" t="s">
         <v>7</v>
@@ -3197,10 +3194,10 @@
         <v>0.5625</v>
       </c>
       <c r="F92" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G92" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H92" t="s">
         <v>13</v>
@@ -3211,7 +3208,7 @@
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B93" t="s">
         <v>7</v>
@@ -3226,10 +3223,10 @@
         <v>0.5625</v>
       </c>
       <c r="F93" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G93" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H93" t="s">
         <v>13</v>
@@ -3240,7 +3237,7 @@
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B94" t="s">
         <v>7</v>
@@ -3255,10 +3252,10 @@
         <v>0.5625</v>
       </c>
       <c r="F94" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G94" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H94" t="s">
         <v>13</v>
@@ -3269,7 +3266,7 @@
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B95" t="s">
         <v>7</v>
@@ -3284,10 +3281,10 @@
         <v>0.5625</v>
       </c>
       <c r="F95" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G95" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H95" t="s">
         <v>13</v>

</xml_diff>